<commit_message>
Fix: Correccion de sub_guest_idx para las etiquetas de las mesas
</commit_message>
<xml_diff>
--- a/RSVP_Guest_List_import.xlsx
+++ b/RSVP_Guest_List_import.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://syngenta-my.sharepoint.com/personal/alejandro_lajnis_syngenta_com/Documents/Ale Personal/IA/RSVP app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="30" documentId="8_{0669B2AD-BB49-463B-A45C-FF5CB10682AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82CDEF07-9FB4-4AB1-96A2-5391036321DF}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{0669B2AD-BB49-463B-A45C-FF5CB10682AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD8AD655-87C5-47BD-9AF7-BC2A03673668}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Guests (Alpha)" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="35">
   <si>
     <t>Email</t>
   </si>
@@ -117,6 +118,27 @@
   </si>
   <si>
     <t>Alicia</t>
+  </si>
+  <si>
+    <t>edad</t>
+  </si>
+  <si>
+    <t>Adulto</t>
+  </si>
+  <si>
+    <t>Niño</t>
+  </si>
+  <si>
+    <t>Teen</t>
+  </si>
+  <si>
+    <t>Bebé</t>
+  </si>
+  <si>
+    <t>Sueyro</t>
+  </si>
+  <si>
+    <t>Matias</t>
   </si>
 </sst>
 </file>
@@ -207,10 +229,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>12700</xdr:colOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>171450</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>44450</xdr:rowOff>
+      <xdr:rowOff>57150</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1714500" cy="781240"/>
     <xdr:sp macro="" textlink="">
@@ -226,7 +248,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5511800" y="44450"/>
+          <a:off x="6896100" y="57150"/>
           <a:ext cx="1714500" cy="781240"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -608,13 +630,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="18.9140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>15</v>
       </c>
@@ -639,8 +661,11 @@
       <c r="H1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>21</v>
       </c>
@@ -665,8 +690,11 @@
       <c r="H2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -691,8 +719,11 @@
       <c r="H3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -717,8 +748,11 @@
       <c r="H4" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -742,6 +776,23 @@
       </c>
       <c r="H5" t="s">
         <v>2</v>
+      </c>
+      <c r="I5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="I6" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -757,6 +808,48 @@
     <ignoredError sqref="C2 C5 E2:H2 C3 E3:F3 C4 E4:F4 E5:F5 D1 H1" numberStoredAsText="1"/>
   </ignoredErrors>
   <drawing r:id="rId5"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{686DBDE1-8816-4579-9A96-971500BCDDBB}">
+          <x14:formula1>
+            <xm:f>Sheet1!$A$1:$A$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>I2:I24</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0DB826B-5DA4-4637-BE7D-4AE258B25B36}">
+  <dimension ref="A1:A4"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>